<commit_message>
Adds renewable diesel lever crudely; need to clean files & fix MDL. Bug: see Transportation Sector Fuel Used[ships,freight,diesel vehicle,petroleum diesel tf]
</commit_message>
<xml_diff>
--- a/InputData/trans/MPoEFUbVT/Max Perc of Each Fuel Usable by Veh Tech.xlsx
+++ b/InputData/trans/MPoEFUbVT/Max Perc of Each Fuel Usable by Veh Tech.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\trans\MPoEFUbVT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\trans\MPoEFUbVT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17FBF57E-9E0A-4861-96FF-003F2EEA3BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8C16FB5-5F07-4EB1-B7F9-C605599A6E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="690" yWindow="1305" windowWidth="23520" windowHeight="15450" firstSheet="67" activeTab="68" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -5393,144 +5393,109 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <f t="shared" ref="B6:AJ6" si="0">max_biogas</f>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="C6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="D6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="F6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="K6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="L6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="M6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="N6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="O6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="Q6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="R6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="S6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="T6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="U6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="V6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="W6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="X6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="Y6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="Z6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AA6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AB6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AC6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AD6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AE6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AF6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AG6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AH6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AI6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AJ6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.25">
@@ -6764,144 +6729,143 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <f t="shared" ref="B7:AJ7" si="0">max_biodsl</f>
-        <v>1</v>
+        <f t="shared" ref="B7:N7" si="0">C7</f>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="D7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="E7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="F7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="G7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="H7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="I7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="J7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="K7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="L7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="M7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="N7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>O7</f>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="O7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" ref="O7:AI7" si="1">P7-0.02</f>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="P7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>9.9999999999999839E-2</v>
       </c>
       <c r="Q7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.11999999999999984</v>
       </c>
       <c r="R7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.13999999999999985</v>
       </c>
       <c r="S7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.15999999999999984</v>
       </c>
       <c r="T7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.17999999999999983</v>
       </c>
       <c r="U7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.19999999999999982</v>
       </c>
       <c r="V7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.21999999999999981</v>
       </c>
       <c r="W7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.2399999999999998</v>
       </c>
       <c r="X7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.25999999999999979</v>
       </c>
       <c r="Y7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.2799999999999998</v>
       </c>
       <c r="Z7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.29999999999999982</v>
       </c>
       <c r="AA7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.31999999999999984</v>
       </c>
       <c r="AB7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.33999999999999986</v>
       </c>
       <c r="AC7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.35999999999999988</v>
       </c>
       <c r="AD7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.37999999999999989</v>
       </c>
       <c r="AE7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.39999999999999991</v>
       </c>
       <c r="AF7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.41999999999999993</v>
       </c>
       <c r="AG7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.43999999999999995</v>
       </c>
       <c r="AH7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.45999999999999996</v>
       </c>
       <c r="AI7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>AJ7-0.02</f>
+        <v>0.48</v>
       </c>
       <c r="AJ7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="8" spans="1:36" x14ac:dyDescent="0.25">
@@ -23389,144 +23353,109 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <f t="shared" ref="B6:AJ6" si="0">max_biogas</f>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="C6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="D6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="F6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="K6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="L6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="M6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="N6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="O6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="Q6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="R6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="S6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="T6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="U6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="V6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="W6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="X6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="Y6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="Z6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AA6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AB6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AC6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AD6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AE6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AF6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AG6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AH6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AI6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="AJ6">
-        <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.25">
@@ -24760,144 +24689,143 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <f t="shared" ref="B7:AJ7" si="0">max_biodsl</f>
-        <v>1</v>
+        <f t="shared" ref="B7:N7" si="0">C7</f>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="D7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="E7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="F7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="G7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="H7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="I7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="J7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="K7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="L7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="M7">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="N7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>O7</f>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="O7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" ref="O7:AI7" si="1">P7-0.02</f>
+        <v>7.9999999999999835E-2</v>
       </c>
       <c r="P7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>9.9999999999999839E-2</v>
       </c>
       <c r="Q7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.11999999999999984</v>
       </c>
       <c r="R7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.13999999999999985</v>
       </c>
       <c r="S7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.15999999999999984</v>
       </c>
       <c r="T7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.17999999999999983</v>
       </c>
       <c r="U7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.19999999999999982</v>
       </c>
       <c r="V7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.21999999999999981</v>
       </c>
       <c r="W7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.2399999999999998</v>
       </c>
       <c r="X7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.25999999999999979</v>
       </c>
       <c r="Y7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.2799999999999998</v>
       </c>
       <c r="Z7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.29999999999999982</v>
       </c>
       <c r="AA7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.31999999999999984</v>
       </c>
       <c r="AB7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.33999999999999986</v>
       </c>
       <c r="AC7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.35999999999999988</v>
       </c>
       <c r="AD7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.37999999999999989</v>
       </c>
       <c r="AE7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.39999999999999991</v>
       </c>
       <c r="AF7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.41999999999999993</v>
       </c>
       <c r="AG7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.43999999999999995</v>
       </c>
       <c r="AH7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>0.45999999999999996</v>
       </c>
       <c r="AI7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f>AJ7-0.02</f>
+        <v>0.48</v>
       </c>
       <c r="AJ7">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="8" spans="1:36" x14ac:dyDescent="0.25">
@@ -33353,128 +33281,116 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <f>'Max Biofuel Blends'!E$14</f>
         <v>0</v>
       </c>
       <c r="F7">
-        <f>'Max Biofuel Blends'!F$14</f>
         <v>0</v>
       </c>
       <c r="G7">
-        <f>'Max Biofuel Blends'!G$14</f>
-        <v>6.6666666666677088E-2</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <f>'Max Biofuel Blends'!H$14</f>
-        <v>0.10000000000000853</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <f>'Max Biofuel Blends'!I$14</f>
-        <v>0.13333333333333997</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <f>'Max Biofuel Blends'!J$14</f>
-        <v>0.1666666666666714</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <f>'Max Biofuel Blends'!K$14</f>
-        <v>0.20000000000000284</v>
+        <v>0</v>
       </c>
       <c r="L7">
-        <f>'Max Biofuel Blends'!L$14</f>
-        <v>0.23333333333333428</v>
+        <v>0</v>
       </c>
       <c r="M7">
-        <f>'Max Biofuel Blends'!M$14</f>
-        <v>0.26666666666666572</v>
+        <v>0</v>
       </c>
       <c r="N7">
-        <f>'Max Biofuel Blends'!N$14</f>
-        <v>0.29999999999999716</v>
+        <v>0</v>
       </c>
       <c r="O7">
-        <f>'Max Biofuel Blends'!O$14</f>
-        <v>0.33333333333334281</v>
+        <v>0</v>
       </c>
       <c r="P7">
-        <f>'Max Biofuel Blends'!P$14</f>
-        <v>0.36666666666667425</v>
+        <f t="shared" ref="O7:AH7" si="0">Q7-0.02</f>
+        <v>1.9999999999999938E-2</v>
       </c>
       <c r="Q7">
-        <f>'Max Biofuel Blends'!Q$14</f>
-        <v>0.40000000000000568</v>
+        <f t="shared" si="0"/>
+        <v>3.9999999999999938E-2</v>
       </c>
       <c r="R7">
-        <f>'Max Biofuel Blends'!R$14</f>
-        <v>0.43333333333333712</v>
+        <f t="shared" si="0"/>
+        <v>5.9999999999999942E-2</v>
       </c>
       <c r="S7">
-        <f>'Max Biofuel Blends'!S$14</f>
-        <v>0.46666666666666856</v>
+        <f t="shared" si="0"/>
+        <v>7.9999999999999946E-2</v>
       </c>
       <c r="T7">
-        <f>'Max Biofuel Blends'!T$14</f>
-        <v>0.5</v>
+        <f t="shared" si="0"/>
+        <v>9.999999999999995E-2</v>
       </c>
       <c r="U7">
-        <f>'Max Biofuel Blends'!U$14</f>
-        <v>0.53333333333333144</v>
+        <f t="shared" si="0"/>
+        <v>0.11999999999999995</v>
       </c>
       <c r="V7">
-        <f>'Max Biofuel Blends'!V$14</f>
-        <v>0.56666666666667709</v>
+        <f t="shared" si="0"/>
+        <v>0.13999999999999996</v>
       </c>
       <c r="W7">
-        <f>'Max Biofuel Blends'!W$14</f>
-        <v>0.60000000000000853</v>
+        <f t="shared" si="0"/>
+        <v>0.15999999999999995</v>
       </c>
       <c r="X7">
-        <f>'Max Biofuel Blends'!X$14</f>
-        <v>0.63333333333333997</v>
+        <f t="shared" si="0"/>
+        <v>0.17999999999999994</v>
       </c>
       <c r="Y7">
-        <f>'Max Biofuel Blends'!Y$14</f>
-        <v>0.6666666666666714</v>
+        <f t="shared" si="0"/>
+        <v>0.19999999999999993</v>
       </c>
       <c r="Z7">
-        <f>'Max Biofuel Blends'!Z$14</f>
-        <v>0.70000000000000284</v>
+        <f t="shared" si="0"/>
+        <v>0.21999999999999992</v>
       </c>
       <c r="AA7">
-        <f>'Max Biofuel Blends'!AA$14</f>
-        <v>0.73333333333333428</v>
+        <f t="shared" si="0"/>
+        <v>0.23999999999999991</v>
       </c>
       <c r="AB7">
-        <f>'Max Biofuel Blends'!AB$14</f>
-        <v>0.76666666666666572</v>
+        <f t="shared" si="0"/>
+        <v>0.2599999999999999</v>
       </c>
       <c r="AC7">
-        <f>'Max Biofuel Blends'!AC$14</f>
-        <v>0.79999999999999716</v>
+        <f t="shared" si="0"/>
+        <v>0.27999999999999992</v>
       </c>
       <c r="AD7">
-        <f>'Max Biofuel Blends'!AD$14</f>
-        <v>0.83333333333334281</v>
+        <f t="shared" si="0"/>
+        <v>0.29999999999999993</v>
       </c>
       <c r="AE7">
-        <f>'Max Biofuel Blends'!AE$14</f>
-        <v>0.86666666666667425</v>
+        <f t="shared" si="0"/>
+        <v>0.31999999999999995</v>
       </c>
       <c r="AF7">
-        <f>'Max Biofuel Blends'!AF$14</f>
-        <v>0.90000000000000568</v>
+        <f t="shared" si="0"/>
+        <v>0.33999999999999997</v>
       </c>
       <c r="AG7">
-        <f>'Max Biofuel Blends'!AG$14</f>
-        <v>0.93333333333333712</v>
+        <f t="shared" si="0"/>
+        <v>0.36</v>
       </c>
       <c r="AH7">
-        <f>'Max Biofuel Blends'!AH$14</f>
-        <v>0.96666666666666856</v>
+        <f>AI7-0.02</f>
+        <v>0.38</v>
       </c>
       <c r="AI7">
-        <f>'Max Biofuel Blends'!AI$14</f>
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.25">
@@ -40624,128 +40540,116 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <f>'Max Biofuel Blends'!E$14</f>
         <v>0</v>
       </c>
       <c r="F7">
-        <f>'Max Biofuel Blends'!F$14</f>
         <v>0</v>
       </c>
       <c r="G7">
-        <f>'Max Biofuel Blends'!G$14</f>
-        <v>6.6666666666677088E-2</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <f>'Max Biofuel Blends'!H$14</f>
-        <v>0.10000000000000853</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <f>'Max Biofuel Blends'!I$14</f>
-        <v>0.13333333333333997</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <f>'Max Biofuel Blends'!J$14</f>
-        <v>0.1666666666666714</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <f>'Max Biofuel Blends'!K$14</f>
-        <v>0.20000000000000284</v>
+        <v>0</v>
       </c>
       <c r="L7">
-        <f>'Max Biofuel Blends'!L$14</f>
-        <v>0.23333333333333428</v>
+        <v>0</v>
       </c>
       <c r="M7">
-        <f>'Max Biofuel Blends'!M$14</f>
-        <v>0.26666666666666572</v>
+        <v>0</v>
       </c>
       <c r="N7">
-        <f>'Max Biofuel Blends'!N$14</f>
-        <v>0.29999999999999716</v>
+        <v>0</v>
       </c>
       <c r="O7">
-        <f>'Max Biofuel Blends'!O$14</f>
-        <v>0.33333333333334281</v>
+        <v>0</v>
       </c>
       <c r="P7">
-        <f>'Max Biofuel Blends'!P$14</f>
-        <v>0.36666666666667425</v>
+        <f t="shared" ref="P7:AI7" si="0">Q7-0.02</f>
+        <v>1.9999999999999938E-2</v>
       </c>
       <c r="Q7">
-        <f>'Max Biofuel Blends'!Q$14</f>
-        <v>0.40000000000000568</v>
+        <f t="shared" si="0"/>
+        <v>3.9999999999999938E-2</v>
       </c>
       <c r="R7">
-        <f>'Max Biofuel Blends'!R$14</f>
-        <v>0.43333333333333712</v>
+        <f t="shared" si="0"/>
+        <v>5.9999999999999942E-2</v>
       </c>
       <c r="S7">
-        <f>'Max Biofuel Blends'!S$14</f>
-        <v>0.46666666666666856</v>
+        <f t="shared" si="0"/>
+        <v>7.9999999999999946E-2</v>
       </c>
       <c r="T7">
-        <f>'Max Biofuel Blends'!T$14</f>
-        <v>0.5</v>
+        <f t="shared" si="0"/>
+        <v>9.999999999999995E-2</v>
       </c>
       <c r="U7">
-        <f>'Max Biofuel Blends'!U$14</f>
-        <v>0.53333333333333144</v>
+        <f t="shared" si="0"/>
+        <v>0.11999999999999995</v>
       </c>
       <c r="V7">
-        <f>'Max Biofuel Blends'!V$14</f>
-        <v>0.56666666666667709</v>
+        <f t="shared" si="0"/>
+        <v>0.13999999999999996</v>
       </c>
       <c r="W7">
-        <f>'Max Biofuel Blends'!W$14</f>
-        <v>0.60000000000000853</v>
+        <f t="shared" si="0"/>
+        <v>0.15999999999999995</v>
       </c>
       <c r="X7">
-        <f>'Max Biofuel Blends'!X$14</f>
-        <v>0.63333333333333997</v>
+        <f t="shared" si="0"/>
+        <v>0.17999999999999994</v>
       </c>
       <c r="Y7">
-        <f>'Max Biofuel Blends'!Y$14</f>
-        <v>0.6666666666666714</v>
+        <f t="shared" si="0"/>
+        <v>0.19999999999999993</v>
       </c>
       <c r="Z7">
-        <f>'Max Biofuel Blends'!Z$14</f>
-        <v>0.70000000000000284</v>
+        <f t="shared" si="0"/>
+        <v>0.21999999999999992</v>
       </c>
       <c r="AA7">
-        <f>'Max Biofuel Blends'!AA$14</f>
-        <v>0.73333333333333428</v>
+        <f t="shared" si="0"/>
+        <v>0.23999999999999991</v>
       </c>
       <c r="AB7">
-        <f>'Max Biofuel Blends'!AB$14</f>
-        <v>0.76666666666666572</v>
+        <f t="shared" si="0"/>
+        <v>0.2599999999999999</v>
       </c>
       <c r="AC7">
-        <f>'Max Biofuel Blends'!AC$14</f>
-        <v>0.79999999999999716</v>
+        <f t="shared" si="0"/>
+        <v>0.27999999999999992</v>
       </c>
       <c r="AD7">
-        <f>'Max Biofuel Blends'!AD$14</f>
-        <v>0.83333333333334281</v>
+        <f t="shared" si="0"/>
+        <v>0.29999999999999993</v>
       </c>
       <c r="AE7">
-        <f>'Max Biofuel Blends'!AE$14</f>
-        <v>0.86666666666667425</v>
+        <f t="shared" si="0"/>
+        <v>0.31999999999999995</v>
       </c>
       <c r="AF7">
-        <f>'Max Biofuel Blends'!AF$14</f>
-        <v>0.90000000000000568</v>
+        <f t="shared" si="0"/>
+        <v>0.33999999999999997</v>
       </c>
       <c r="AG7">
-        <f>'Max Biofuel Blends'!AG$14</f>
-        <v>0.93333333333333712</v>
+        <f t="shared" si="0"/>
+        <v>0.36</v>
       </c>
       <c r="AH7">
-        <f>'Max Biofuel Blends'!AH$14</f>
-        <v>0.96666666666666856</v>
+        <f>AI7-0.02</f>
+        <v>0.38</v>
       </c>
       <c r="AI7">
-        <f>'Max Biofuel Blends'!AI$14</f>
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.25">
@@ -61234,140 +61138,125 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <f>'Max Biofuel Blends'!B$14</f>
         <v>0</v>
       </c>
       <c r="C7">
-        <f>'Max Biofuel Blends'!C$14</f>
         <v>0</v>
       </c>
       <c r="D7">
-        <f>'Max Biofuel Blends'!D$14</f>
         <v>0</v>
       </c>
       <c r="E7">
-        <f>'Max Biofuel Blends'!E$14</f>
         <v>0</v>
       </c>
       <c r="F7">
-        <f>'Max Biofuel Blends'!F$14</f>
         <v>0</v>
       </c>
       <c r="G7">
-        <f>'Max Biofuel Blends'!G$14</f>
-        <v>6.6666666666677088E-2</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <f>'Max Biofuel Blends'!H$14</f>
-        <v>0.10000000000000853</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <f>'Max Biofuel Blends'!I$14</f>
-        <v>0.13333333333333997</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <f>'Max Biofuel Blends'!J$14</f>
-        <v>0.1666666666666714</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <f>'Max Biofuel Blends'!K$14</f>
-        <v>0.20000000000000284</v>
+        <v>0</v>
       </c>
       <c r="L7">
-        <f>'Max Biofuel Blends'!L$14</f>
-        <v>0.23333333333333428</v>
+        <v>0</v>
       </c>
       <c r="M7">
-        <f>'Max Biofuel Blends'!M$14</f>
-        <v>0.26666666666666572</v>
+        <v>0</v>
       </c>
       <c r="N7">
-        <f>'Max Biofuel Blends'!N$14</f>
-        <v>0.29999999999999716</v>
+        <v>0</v>
       </c>
       <c r="O7">
-        <f>'Max Biofuel Blends'!O$14</f>
-        <v>0.33333333333334281</v>
+        <v>0</v>
       </c>
       <c r="P7">
-        <f>'Max Biofuel Blends'!P$14</f>
-        <v>0.36666666666667425</v>
+        <f t="shared" ref="O7:AH7" si="0">Q7-0.02</f>
+        <v>1.9999999999999938E-2</v>
       </c>
       <c r="Q7">
-        <f>'Max Biofuel Blends'!Q$14</f>
-        <v>0.40000000000000568</v>
+        <f t="shared" si="0"/>
+        <v>3.9999999999999938E-2</v>
       </c>
       <c r="R7">
-        <f>'Max Biofuel Blends'!R$14</f>
-        <v>0.43333333333333712</v>
+        <f t="shared" si="0"/>
+        <v>5.9999999999999942E-2</v>
       </c>
       <c r="S7">
-        <f>'Max Biofuel Blends'!S$14</f>
-        <v>0.46666666666666856</v>
+        <f t="shared" si="0"/>
+        <v>7.9999999999999946E-2</v>
       </c>
       <c r="T7">
-        <f>'Max Biofuel Blends'!T$14</f>
-        <v>0.5</v>
+        <f t="shared" si="0"/>
+        <v>9.999999999999995E-2</v>
       </c>
       <c r="U7">
-        <f>'Max Biofuel Blends'!U$14</f>
-        <v>0.53333333333333144</v>
+        <f t="shared" si="0"/>
+        <v>0.11999999999999995</v>
       </c>
       <c r="V7">
-        <f>'Max Biofuel Blends'!V$14</f>
-        <v>0.56666666666667709</v>
+        <f t="shared" si="0"/>
+        <v>0.13999999999999996</v>
       </c>
       <c r="W7">
-        <f>'Max Biofuel Blends'!W$14</f>
-        <v>0.60000000000000853</v>
+        <f t="shared" si="0"/>
+        <v>0.15999999999999995</v>
       </c>
       <c r="X7">
-        <f>'Max Biofuel Blends'!X$14</f>
-        <v>0.63333333333333997</v>
+        <f t="shared" si="0"/>
+        <v>0.17999999999999994</v>
       </c>
       <c r="Y7">
-        <f>'Max Biofuel Blends'!Y$14</f>
-        <v>0.6666666666666714</v>
+        <f t="shared" si="0"/>
+        <v>0.19999999999999993</v>
       </c>
       <c r="Z7">
-        <f>'Max Biofuel Blends'!Z$14</f>
-        <v>0.70000000000000284</v>
+        <f t="shared" si="0"/>
+        <v>0.21999999999999992</v>
       </c>
       <c r="AA7">
-        <f>'Max Biofuel Blends'!AA$14</f>
-        <v>0.73333333333333428</v>
+        <f t="shared" si="0"/>
+        <v>0.23999999999999991</v>
       </c>
       <c r="AB7">
-        <f>'Max Biofuel Blends'!AB$14</f>
-        <v>0.76666666666666572</v>
+        <f t="shared" si="0"/>
+        <v>0.2599999999999999</v>
       </c>
       <c r="AC7">
-        <f>'Max Biofuel Blends'!AC$14</f>
-        <v>0.79999999999999716</v>
+        <f t="shared" si="0"/>
+        <v>0.27999999999999992</v>
       </c>
       <c r="AD7">
-        <f>'Max Biofuel Blends'!AD$14</f>
-        <v>0.83333333333334281</v>
+        <f t="shared" si="0"/>
+        <v>0.29999999999999993</v>
       </c>
       <c r="AE7">
-        <f>'Max Biofuel Blends'!AE$14</f>
-        <v>0.86666666666667425</v>
+        <f t="shared" si="0"/>
+        <v>0.31999999999999995</v>
       </c>
       <c r="AF7">
-        <f>'Max Biofuel Blends'!AF$14</f>
-        <v>0.90000000000000568</v>
+        <f t="shared" si="0"/>
+        <v>0.33999999999999997</v>
       </c>
       <c r="AG7">
-        <f>'Max Biofuel Blends'!AG$14</f>
-        <v>0.93333333333333712</v>
+        <f t="shared" si="0"/>
+        <v>0.36</v>
       </c>
       <c r="AH7">
-        <f>'Max Biofuel Blends'!AH$14</f>
-        <v>0.96666666666666856</v>
+        <f>AI7-0.02</f>
+        <v>0.38</v>
       </c>
       <c r="AI7">
-        <f>'Max Biofuel Blends'!AI$14</f>
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.25">
@@ -67279,140 +67168,125 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <f>'Max Biofuel Blends'!B$17</f>
         <v>0</v>
       </c>
       <c r="C7">
-        <f>'Max Biofuel Blends'!C$17</f>
         <v>0</v>
       </c>
       <c r="D7">
-        <f>'Max Biofuel Blends'!D$17</f>
         <v>0</v>
       </c>
       <c r="E7">
-        <f>'Max Biofuel Blends'!E$17</f>
         <v>0</v>
       </c>
       <c r="F7">
-        <f>'Max Biofuel Blends'!F$17</f>
         <v>0</v>
       </c>
       <c r="G7">
-        <f>'Max Biofuel Blends'!G$17</f>
-        <v>3.9999999999992042E-2</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <f>'Max Biofuel Blends'!H$17</f>
-        <v>5.9999999999995168E-2</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <f>'Max Biofuel Blends'!I$17</f>
-        <v>7.9999999999998295E-2</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <f>'Max Biofuel Blends'!J$17</f>
-        <v>9.9999999999994316E-2</v>
+        <v>0</v>
       </c>
       <c r="K7">
-        <f>'Max Biofuel Blends'!K$17</f>
-        <v>0.11999999999999744</v>
+        <v>0</v>
       </c>
       <c r="L7">
-        <f>'Max Biofuel Blends'!L$17</f>
-        <v>0.13999999999999346</v>
+        <v>0</v>
       </c>
       <c r="M7">
-        <f>'Max Biofuel Blends'!M$17</f>
-        <v>0.15999999999999659</v>
+        <v>0</v>
       </c>
       <c r="N7">
-        <f>'Max Biofuel Blends'!N$17</f>
-        <v>0.17999999999999261</v>
+        <v>0</v>
       </c>
       <c r="O7">
-        <f>'Max Biofuel Blends'!O$17</f>
-        <v>0.19999999999999574</v>
+        <v>0</v>
       </c>
       <c r="P7">
-        <f>'Max Biofuel Blends'!P$17</f>
-        <v>0.21999999999999176</v>
+        <f t="shared" ref="P7:AH7" si="0">Q7-0.02</f>
+        <v>1.9999999999999938E-2</v>
       </c>
       <c r="Q7">
-        <f>'Max Biofuel Blends'!Q$17</f>
-        <v>0.23999999999999488</v>
+        <f t="shared" si="0"/>
+        <v>3.9999999999999938E-2</v>
       </c>
       <c r="R7">
-        <f>'Max Biofuel Blends'!R$17</f>
-        <v>0.25999999999999801</v>
+        <f t="shared" si="0"/>
+        <v>5.9999999999999942E-2</v>
       </c>
       <c r="S7">
-        <f>'Max Biofuel Blends'!S$17</f>
-        <v>0.27999999999999403</v>
+        <f t="shared" si="0"/>
+        <v>7.9999999999999946E-2</v>
       </c>
       <c r="T7">
-        <f>'Max Biofuel Blends'!T$17</f>
-        <v>0.29999999999999716</v>
+        <f t="shared" si="0"/>
+        <v>9.999999999999995E-2</v>
       </c>
       <c r="U7">
-        <f>'Max Biofuel Blends'!U$17</f>
-        <v>0.31999999999999318</v>
+        <f t="shared" si="0"/>
+        <v>0.11999999999999995</v>
       </c>
       <c r="V7">
-        <f>'Max Biofuel Blends'!V$17</f>
-        <v>0.33999999999999631</v>
+        <f t="shared" si="0"/>
+        <v>0.13999999999999996</v>
       </c>
       <c r="W7">
-        <f>'Max Biofuel Blends'!W$17</f>
-        <v>0.35999999999999233</v>
+        <f t="shared" si="0"/>
+        <v>0.15999999999999995</v>
       </c>
       <c r="X7">
-        <f>'Max Biofuel Blends'!X$17</f>
-        <v>0.37999999999999545</v>
+        <f t="shared" si="0"/>
+        <v>0.17999999999999994</v>
       </c>
       <c r="Y7">
-        <f>'Max Biofuel Blends'!Y$17</f>
-        <v>0.39999999999999858</v>
+        <f t="shared" si="0"/>
+        <v>0.19999999999999993</v>
       </c>
       <c r="Z7">
-        <f>'Max Biofuel Blends'!Z$17</f>
-        <v>0.4199999999999946</v>
+        <f t="shared" si="0"/>
+        <v>0.21999999999999992</v>
       </c>
       <c r="AA7">
-        <f>'Max Biofuel Blends'!AA$17</f>
-        <v>0.43999999999999773</v>
+        <f t="shared" si="0"/>
+        <v>0.23999999999999991</v>
       </c>
       <c r="AB7">
-        <f>'Max Biofuel Blends'!AB$17</f>
-        <v>0.45999999999999375</v>
+        <f t="shared" si="0"/>
+        <v>0.2599999999999999</v>
       </c>
       <c r="AC7">
-        <f>'Max Biofuel Blends'!AC$17</f>
-        <v>0.47999999999999687</v>
+        <f t="shared" si="0"/>
+        <v>0.27999999999999992</v>
       </c>
       <c r="AD7">
-        <f>'Max Biofuel Blends'!AD$17</f>
-        <v>0.49999999999999289</v>
+        <f t="shared" si="0"/>
+        <v>0.29999999999999993</v>
       </c>
       <c r="AE7">
-        <f>'Max Biofuel Blends'!AE$17</f>
-        <v>0.51999999999999602</v>
+        <f t="shared" si="0"/>
+        <v>0.31999999999999995</v>
       </c>
       <c r="AF7">
-        <f>'Max Biofuel Blends'!AF$17</f>
-        <v>0.53999999999999204</v>
+        <f t="shared" si="0"/>
+        <v>0.33999999999999997</v>
       </c>
       <c r="AG7">
-        <f>'Max Biofuel Blends'!AG$17</f>
-        <v>0.55999999999999517</v>
+        <f t="shared" si="0"/>
+        <v>0.36</v>
       </c>
       <c r="AH7">
-        <f>'Max Biofuel Blends'!AH$17</f>
-        <v>0.57999999999999829</v>
+        <f>AI7-0.02</f>
+        <v>0.38</v>
       </c>
       <c r="AI7">
-        <f>'Max Biofuel Blends'!AI$17</f>
-        <v>0.59999999999999432</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Reverses changes to MPoEFUbVT from prior commit & builds a non-BAU version to allow differing policy scenario without modifying BAU; adopts into US Climate Ambition scenario to represent drop-in renewable diesel credits
</commit_message>
<xml_diff>
--- a/InputData/trans/MPoEFUbVT/Max Perc of Each Fuel Usable by Veh Tech.xlsx
+++ b/InputData/trans/MPoEFUbVT/Max Perc of Each Fuel Usable by Veh Tech.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\trans\MPoEFUbVT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8C16FB5-5F07-4EB1-B7F9-C605599A6E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{036B868E-71DA-4EB8-BD7B-BEB6F04D77CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="690" yWindow="1305" windowWidth="23520" windowHeight="15450" firstSheet="67" activeTab="68" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2820" yWindow="1110" windowWidth="23520" windowHeight="15450" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -5393,109 +5393,144 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <f t="shared" ref="B6:AJ6" si="0">max_biogas</f>
+        <v>0.15</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="J6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="L6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="M6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="Q6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="R6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="T6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="U6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="V6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="W6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="X6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="Y6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="Z6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AA6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AB6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AC6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AD6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AE6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AF6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AG6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AH6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AI6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AJ6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.25">
@@ -6729,143 +6764,144 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <f t="shared" ref="B7:N7" si="0">C7</f>
-        <v>7.9999999999999835E-2</v>
+        <f t="shared" ref="B7:AJ7" si="0">max_biodsl</f>
+        <v>1</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="D7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="E7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="F7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="G7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="H7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="I7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="J7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="K7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="L7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="M7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="N7">
-        <f>O7</f>
-        <v>7.9999999999999835E-2</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="O7">
-        <f t="shared" ref="O7:AI7" si="1">P7-0.02</f>
-        <v>7.9999999999999835E-2</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="P7">
-        <f t="shared" si="1"/>
-        <v>9.9999999999999839E-2</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="Q7">
-        <f t="shared" si="1"/>
-        <v>0.11999999999999984</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="R7">
-        <f t="shared" si="1"/>
-        <v>0.13999999999999985</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="S7">
-        <f t="shared" si="1"/>
-        <v>0.15999999999999984</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="T7">
-        <f t="shared" si="1"/>
-        <v>0.17999999999999983</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="U7">
-        <f t="shared" si="1"/>
-        <v>0.19999999999999982</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="V7">
-        <f t="shared" si="1"/>
-        <v>0.21999999999999981</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="W7">
-        <f t="shared" si="1"/>
-        <v>0.2399999999999998</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="X7">
-        <f t="shared" si="1"/>
-        <v>0.25999999999999979</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="Y7">
-        <f t="shared" si="1"/>
-        <v>0.2799999999999998</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="Z7">
-        <f t="shared" si="1"/>
-        <v>0.29999999999999982</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AA7">
-        <f t="shared" si="1"/>
-        <v>0.31999999999999984</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AB7">
-        <f t="shared" si="1"/>
-        <v>0.33999999999999986</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AC7">
-        <f t="shared" si="1"/>
-        <v>0.35999999999999988</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AD7">
-        <f t="shared" si="1"/>
-        <v>0.37999999999999989</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AE7">
-        <f t="shared" si="1"/>
-        <v>0.39999999999999991</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AF7">
-        <f t="shared" si="1"/>
-        <v>0.41999999999999993</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AG7">
-        <f t="shared" si="1"/>
-        <v>0.43999999999999995</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AH7">
-        <f t="shared" si="1"/>
-        <v>0.45999999999999996</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AI7">
-        <f>AJ7-0.02</f>
-        <v>0.48</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AJ7">
-        <v>0.5</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:36" x14ac:dyDescent="0.25">
@@ -23353,109 +23389,144 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <f t="shared" ref="B6:AJ6" si="0">max_biogas</f>
+        <v>0.15</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="J6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="L6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="M6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="Q6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="R6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="T6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="U6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="V6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="W6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="X6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="Y6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="Z6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AA6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AB6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AC6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AD6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AE6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AF6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AG6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AH6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AI6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
       <c r="AJ6">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>0.15</v>
       </c>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.25">
@@ -24689,143 +24760,144 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <f t="shared" ref="B7:N7" si="0">C7</f>
-        <v>7.9999999999999835E-2</v>
+        <f t="shared" ref="B7:AJ7" si="0">max_biodsl</f>
+        <v>1</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="D7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="E7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="F7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="G7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="H7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="I7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="J7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="K7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="L7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="M7">
         <f t="shared" si="0"/>
-        <v>7.9999999999999835E-2</v>
+        <v>1</v>
       </c>
       <c r="N7">
-        <f>O7</f>
-        <v>7.9999999999999835E-2</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="O7">
-        <f t="shared" ref="O7:AI7" si="1">P7-0.02</f>
-        <v>7.9999999999999835E-2</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="P7">
-        <f t="shared" si="1"/>
-        <v>9.9999999999999839E-2</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="Q7">
-        <f t="shared" si="1"/>
-        <v>0.11999999999999984</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="R7">
-        <f t="shared" si="1"/>
-        <v>0.13999999999999985</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="S7">
-        <f t="shared" si="1"/>
-        <v>0.15999999999999984</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="T7">
-        <f t="shared" si="1"/>
-        <v>0.17999999999999983</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="U7">
-        <f t="shared" si="1"/>
-        <v>0.19999999999999982</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="V7">
-        <f t="shared" si="1"/>
-        <v>0.21999999999999981</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="W7">
-        <f t="shared" si="1"/>
-        <v>0.2399999999999998</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="X7">
-        <f t="shared" si="1"/>
-        <v>0.25999999999999979</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="Y7">
-        <f t="shared" si="1"/>
-        <v>0.2799999999999998</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="Z7">
-        <f t="shared" si="1"/>
-        <v>0.29999999999999982</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AA7">
-        <f t="shared" si="1"/>
-        <v>0.31999999999999984</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AB7">
-        <f t="shared" si="1"/>
-        <v>0.33999999999999986</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AC7">
-        <f t="shared" si="1"/>
-        <v>0.35999999999999988</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AD7">
-        <f t="shared" si="1"/>
-        <v>0.37999999999999989</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AE7">
-        <f t="shared" si="1"/>
-        <v>0.39999999999999991</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AF7">
-        <f t="shared" si="1"/>
-        <v>0.41999999999999993</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AG7">
-        <f t="shared" si="1"/>
-        <v>0.43999999999999995</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AH7">
-        <f t="shared" si="1"/>
-        <v>0.45999999999999996</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AI7">
-        <f>AJ7-0.02</f>
-        <v>0.48</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="AJ7">
-        <v>0.5</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:36" x14ac:dyDescent="0.25">
@@ -33281,116 +33353,128 @@
         <v>0</v>
       </c>
       <c r="E7">
+        <f>'Max Biofuel Blends'!E$14</f>
         <v>0</v>
       </c>
       <c r="F7">
+        <f>'Max Biofuel Blends'!F$14</f>
         <v>0</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!G$14</f>
+        <v>6.6666666666677088E-2</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!H$14</f>
+        <v>0.10000000000000853</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!I$14</f>
+        <v>0.13333333333333997</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!J$14</f>
+        <v>0.1666666666666714</v>
       </c>
       <c r="K7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!K$14</f>
+        <v>0.20000000000000284</v>
       </c>
       <c r="L7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!L$14</f>
+        <v>0.23333333333333428</v>
       </c>
       <c r="M7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!M$14</f>
+        <v>0.26666666666666572</v>
       </c>
       <c r="N7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!N$14</f>
+        <v>0.29999999999999716</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!O$14</f>
+        <v>0.33333333333334281</v>
       </c>
       <c r="P7">
-        <f t="shared" ref="O7:AH7" si="0">Q7-0.02</f>
-        <v>1.9999999999999938E-2</v>
+        <f>'Max Biofuel Blends'!P$14</f>
+        <v>0.36666666666667425</v>
       </c>
       <c r="Q7">
-        <f t="shared" si="0"/>
-        <v>3.9999999999999938E-2</v>
+        <f>'Max Biofuel Blends'!Q$14</f>
+        <v>0.40000000000000568</v>
       </c>
       <c r="R7">
-        <f t="shared" si="0"/>
-        <v>5.9999999999999942E-2</v>
+        <f>'Max Biofuel Blends'!R$14</f>
+        <v>0.43333333333333712</v>
       </c>
       <c r="S7">
-        <f t="shared" si="0"/>
-        <v>7.9999999999999946E-2</v>
+        <f>'Max Biofuel Blends'!S$14</f>
+        <v>0.46666666666666856</v>
       </c>
       <c r="T7">
-        <f t="shared" si="0"/>
-        <v>9.999999999999995E-2</v>
+        <f>'Max Biofuel Blends'!T$14</f>
+        <v>0.5</v>
       </c>
       <c r="U7">
-        <f t="shared" si="0"/>
-        <v>0.11999999999999995</v>
+        <f>'Max Biofuel Blends'!U$14</f>
+        <v>0.53333333333333144</v>
       </c>
       <c r="V7">
-        <f t="shared" si="0"/>
-        <v>0.13999999999999996</v>
+        <f>'Max Biofuel Blends'!V$14</f>
+        <v>0.56666666666667709</v>
       </c>
       <c r="W7">
-        <f t="shared" si="0"/>
-        <v>0.15999999999999995</v>
+        <f>'Max Biofuel Blends'!W$14</f>
+        <v>0.60000000000000853</v>
       </c>
       <c r="X7">
-        <f t="shared" si="0"/>
-        <v>0.17999999999999994</v>
+        <f>'Max Biofuel Blends'!X$14</f>
+        <v>0.63333333333333997</v>
       </c>
       <c r="Y7">
-        <f t="shared" si="0"/>
-        <v>0.19999999999999993</v>
+        <f>'Max Biofuel Blends'!Y$14</f>
+        <v>0.6666666666666714</v>
       </c>
       <c r="Z7">
-        <f t="shared" si="0"/>
-        <v>0.21999999999999992</v>
+        <f>'Max Biofuel Blends'!Z$14</f>
+        <v>0.70000000000000284</v>
       </c>
       <c r="AA7">
-        <f t="shared" si="0"/>
-        <v>0.23999999999999991</v>
+        <f>'Max Biofuel Blends'!AA$14</f>
+        <v>0.73333333333333428</v>
       </c>
       <c r="AB7">
-        <f t="shared" si="0"/>
-        <v>0.2599999999999999</v>
+        <f>'Max Biofuel Blends'!AB$14</f>
+        <v>0.76666666666666572</v>
       </c>
       <c r="AC7">
-        <f t="shared" si="0"/>
-        <v>0.27999999999999992</v>
+        <f>'Max Biofuel Blends'!AC$14</f>
+        <v>0.79999999999999716</v>
       </c>
       <c r="AD7">
-        <f t="shared" si="0"/>
-        <v>0.29999999999999993</v>
+        <f>'Max Biofuel Blends'!AD$14</f>
+        <v>0.83333333333334281</v>
       </c>
       <c r="AE7">
-        <f t="shared" si="0"/>
-        <v>0.31999999999999995</v>
+        <f>'Max Biofuel Blends'!AE$14</f>
+        <v>0.86666666666667425</v>
       </c>
       <c r="AF7">
-        <f t="shared" si="0"/>
-        <v>0.33999999999999997</v>
+        <f>'Max Biofuel Blends'!AF$14</f>
+        <v>0.90000000000000568</v>
       </c>
       <c r="AG7">
-        <f t="shared" si="0"/>
-        <v>0.36</v>
+        <f>'Max Biofuel Blends'!AG$14</f>
+        <v>0.93333333333333712</v>
       </c>
       <c r="AH7">
-        <f>AI7-0.02</f>
-        <v>0.38</v>
+        <f>'Max Biofuel Blends'!AH$14</f>
+        <v>0.96666666666666856</v>
       </c>
       <c r="AI7">
-        <v>0.4</v>
+        <f>'Max Biofuel Blends'!AI$14</f>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.25">
@@ -40540,116 +40624,128 @@
         <v>0</v>
       </c>
       <c r="E7">
+        <f>'Max Biofuel Blends'!E$14</f>
         <v>0</v>
       </c>
       <c r="F7">
+        <f>'Max Biofuel Blends'!F$14</f>
         <v>0</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!G$14</f>
+        <v>6.6666666666677088E-2</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!H$14</f>
+        <v>0.10000000000000853</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!I$14</f>
+        <v>0.13333333333333997</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!J$14</f>
+        <v>0.1666666666666714</v>
       </c>
       <c r="K7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!K$14</f>
+        <v>0.20000000000000284</v>
       </c>
       <c r="L7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!L$14</f>
+        <v>0.23333333333333428</v>
       </c>
       <c r="M7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!M$14</f>
+        <v>0.26666666666666572</v>
       </c>
       <c r="N7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!N$14</f>
+        <v>0.29999999999999716</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!O$14</f>
+        <v>0.33333333333334281</v>
       </c>
       <c r="P7">
-        <f t="shared" ref="P7:AI7" si="0">Q7-0.02</f>
-        <v>1.9999999999999938E-2</v>
+        <f>'Max Biofuel Blends'!P$14</f>
+        <v>0.36666666666667425</v>
       </c>
       <c r="Q7">
-        <f t="shared" si="0"/>
-        <v>3.9999999999999938E-2</v>
+        <f>'Max Biofuel Blends'!Q$14</f>
+        <v>0.40000000000000568</v>
       </c>
       <c r="R7">
-        <f t="shared" si="0"/>
-        <v>5.9999999999999942E-2</v>
+        <f>'Max Biofuel Blends'!R$14</f>
+        <v>0.43333333333333712</v>
       </c>
       <c r="S7">
-        <f t="shared" si="0"/>
-        <v>7.9999999999999946E-2</v>
+        <f>'Max Biofuel Blends'!S$14</f>
+        <v>0.46666666666666856</v>
       </c>
       <c r="T7">
-        <f t="shared" si="0"/>
-        <v>9.999999999999995E-2</v>
+        <f>'Max Biofuel Blends'!T$14</f>
+        <v>0.5</v>
       </c>
       <c r="U7">
-        <f t="shared" si="0"/>
-        <v>0.11999999999999995</v>
+        <f>'Max Biofuel Blends'!U$14</f>
+        <v>0.53333333333333144</v>
       </c>
       <c r="V7">
-        <f t="shared" si="0"/>
-        <v>0.13999999999999996</v>
+        <f>'Max Biofuel Blends'!V$14</f>
+        <v>0.56666666666667709</v>
       </c>
       <c r="W7">
-        <f t="shared" si="0"/>
-        <v>0.15999999999999995</v>
+        <f>'Max Biofuel Blends'!W$14</f>
+        <v>0.60000000000000853</v>
       </c>
       <c r="X7">
-        <f t="shared" si="0"/>
-        <v>0.17999999999999994</v>
+        <f>'Max Biofuel Blends'!X$14</f>
+        <v>0.63333333333333997</v>
       </c>
       <c r="Y7">
-        <f t="shared" si="0"/>
-        <v>0.19999999999999993</v>
+        <f>'Max Biofuel Blends'!Y$14</f>
+        <v>0.6666666666666714</v>
       </c>
       <c r="Z7">
-        <f t="shared" si="0"/>
-        <v>0.21999999999999992</v>
+        <f>'Max Biofuel Blends'!Z$14</f>
+        <v>0.70000000000000284</v>
       </c>
       <c r="AA7">
-        <f t="shared" si="0"/>
-        <v>0.23999999999999991</v>
+        <f>'Max Biofuel Blends'!AA$14</f>
+        <v>0.73333333333333428</v>
       </c>
       <c r="AB7">
-        <f t="shared" si="0"/>
-        <v>0.2599999999999999</v>
+        <f>'Max Biofuel Blends'!AB$14</f>
+        <v>0.76666666666666572</v>
       </c>
       <c r="AC7">
-        <f t="shared" si="0"/>
-        <v>0.27999999999999992</v>
+        <f>'Max Biofuel Blends'!AC$14</f>
+        <v>0.79999999999999716</v>
       </c>
       <c r="AD7">
-        <f t="shared" si="0"/>
-        <v>0.29999999999999993</v>
+        <f>'Max Biofuel Blends'!AD$14</f>
+        <v>0.83333333333334281</v>
       </c>
       <c r="AE7">
-        <f t="shared" si="0"/>
-        <v>0.31999999999999995</v>
+        <f>'Max Biofuel Blends'!AE$14</f>
+        <v>0.86666666666667425</v>
       </c>
       <c r="AF7">
-        <f t="shared" si="0"/>
-        <v>0.33999999999999997</v>
+        <f>'Max Biofuel Blends'!AF$14</f>
+        <v>0.90000000000000568</v>
       </c>
       <c r="AG7">
-        <f t="shared" si="0"/>
-        <v>0.36</v>
+        <f>'Max Biofuel Blends'!AG$14</f>
+        <v>0.93333333333333712</v>
       </c>
       <c r="AH7">
-        <f>AI7-0.02</f>
-        <v>0.38</v>
+        <f>'Max Biofuel Blends'!AH$14</f>
+        <v>0.96666666666666856</v>
       </c>
       <c r="AI7">
-        <v>0.4</v>
+        <f>'Max Biofuel Blends'!AI$14</f>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.25">
@@ -61138,125 +61234,140 @@
         <v>8</v>
       </c>
       <c r="B7">
+        <f>'Max Biofuel Blends'!B$14</f>
         <v>0</v>
       </c>
       <c r="C7">
+        <f>'Max Biofuel Blends'!C$14</f>
         <v>0</v>
       </c>
       <c r="D7">
+        <f>'Max Biofuel Blends'!D$14</f>
         <v>0</v>
       </c>
       <c r="E7">
+        <f>'Max Biofuel Blends'!E$14</f>
         <v>0</v>
       </c>
       <c r="F7">
+        <f>'Max Biofuel Blends'!F$14</f>
         <v>0</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!G$14</f>
+        <v>6.6666666666677088E-2</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!H$14</f>
+        <v>0.10000000000000853</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!I$14</f>
+        <v>0.13333333333333997</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!J$14</f>
+        <v>0.1666666666666714</v>
       </c>
       <c r="K7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!K$14</f>
+        <v>0.20000000000000284</v>
       </c>
       <c r="L7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!L$14</f>
+        <v>0.23333333333333428</v>
       </c>
       <c r="M7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!M$14</f>
+        <v>0.26666666666666572</v>
       </c>
       <c r="N7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!N$14</f>
+        <v>0.29999999999999716</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!O$14</f>
+        <v>0.33333333333334281</v>
       </c>
       <c r="P7">
-        <f t="shared" ref="O7:AH7" si="0">Q7-0.02</f>
-        <v>1.9999999999999938E-2</v>
+        <f>'Max Biofuel Blends'!P$14</f>
+        <v>0.36666666666667425</v>
       </c>
       <c r="Q7">
-        <f t="shared" si="0"/>
-        <v>3.9999999999999938E-2</v>
+        <f>'Max Biofuel Blends'!Q$14</f>
+        <v>0.40000000000000568</v>
       </c>
       <c r="R7">
-        <f t="shared" si="0"/>
-        <v>5.9999999999999942E-2</v>
+        <f>'Max Biofuel Blends'!R$14</f>
+        <v>0.43333333333333712</v>
       </c>
       <c r="S7">
-        <f t="shared" si="0"/>
-        <v>7.9999999999999946E-2</v>
+        <f>'Max Biofuel Blends'!S$14</f>
+        <v>0.46666666666666856</v>
       </c>
       <c r="T7">
-        <f t="shared" si="0"/>
-        <v>9.999999999999995E-2</v>
+        <f>'Max Biofuel Blends'!T$14</f>
+        <v>0.5</v>
       </c>
       <c r="U7">
-        <f t="shared" si="0"/>
-        <v>0.11999999999999995</v>
+        <f>'Max Biofuel Blends'!U$14</f>
+        <v>0.53333333333333144</v>
       </c>
       <c r="V7">
-        <f t="shared" si="0"/>
-        <v>0.13999999999999996</v>
+        <f>'Max Biofuel Blends'!V$14</f>
+        <v>0.56666666666667709</v>
       </c>
       <c r="W7">
-        <f t="shared" si="0"/>
-        <v>0.15999999999999995</v>
+        <f>'Max Biofuel Blends'!W$14</f>
+        <v>0.60000000000000853</v>
       </c>
       <c r="X7">
-        <f t="shared" si="0"/>
-        <v>0.17999999999999994</v>
+        <f>'Max Biofuel Blends'!X$14</f>
+        <v>0.63333333333333997</v>
       </c>
       <c r="Y7">
-        <f t="shared" si="0"/>
-        <v>0.19999999999999993</v>
+        <f>'Max Biofuel Blends'!Y$14</f>
+        <v>0.6666666666666714</v>
       </c>
       <c r="Z7">
-        <f t="shared" si="0"/>
-        <v>0.21999999999999992</v>
+        <f>'Max Biofuel Blends'!Z$14</f>
+        <v>0.70000000000000284</v>
       </c>
       <c r="AA7">
-        <f t="shared" si="0"/>
-        <v>0.23999999999999991</v>
+        <f>'Max Biofuel Blends'!AA$14</f>
+        <v>0.73333333333333428</v>
       </c>
       <c r="AB7">
-        <f t="shared" si="0"/>
-        <v>0.2599999999999999</v>
+        <f>'Max Biofuel Blends'!AB$14</f>
+        <v>0.76666666666666572</v>
       </c>
       <c r="AC7">
-        <f t="shared" si="0"/>
-        <v>0.27999999999999992</v>
+        <f>'Max Biofuel Blends'!AC$14</f>
+        <v>0.79999999999999716</v>
       </c>
       <c r="AD7">
-        <f t="shared" si="0"/>
-        <v>0.29999999999999993</v>
+        <f>'Max Biofuel Blends'!AD$14</f>
+        <v>0.83333333333334281</v>
       </c>
       <c r="AE7">
-        <f t="shared" si="0"/>
-        <v>0.31999999999999995</v>
+        <f>'Max Biofuel Blends'!AE$14</f>
+        <v>0.86666666666667425</v>
       </c>
       <c r="AF7">
-        <f t="shared" si="0"/>
-        <v>0.33999999999999997</v>
+        <f>'Max Biofuel Blends'!AF$14</f>
+        <v>0.90000000000000568</v>
       </c>
       <c r="AG7">
-        <f t="shared" si="0"/>
-        <v>0.36</v>
+        <f>'Max Biofuel Blends'!AG$14</f>
+        <v>0.93333333333333712</v>
       </c>
       <c r="AH7">
-        <f>AI7-0.02</f>
-        <v>0.38</v>
+        <f>'Max Biofuel Blends'!AH$14</f>
+        <v>0.96666666666666856</v>
       </c>
       <c r="AI7">
-        <v>0.4</v>
+        <f>'Max Biofuel Blends'!AI$14</f>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.25">
@@ -67168,125 +67279,140 @@
         <v>8</v>
       </c>
       <c r="B7">
+        <f>'Max Biofuel Blends'!B$17</f>
         <v>0</v>
       </c>
       <c r="C7">
+        <f>'Max Biofuel Blends'!C$17</f>
         <v>0</v>
       </c>
       <c r="D7">
+        <f>'Max Biofuel Blends'!D$17</f>
         <v>0</v>
       </c>
       <c r="E7">
+        <f>'Max Biofuel Blends'!E$17</f>
         <v>0</v>
       </c>
       <c r="F7">
+        <f>'Max Biofuel Blends'!F$17</f>
         <v>0</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!G$17</f>
+        <v>3.9999999999992042E-2</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!H$17</f>
+        <v>5.9999999999995168E-2</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!I$17</f>
+        <v>7.9999999999998295E-2</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!J$17</f>
+        <v>9.9999999999994316E-2</v>
       </c>
       <c r="K7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!K$17</f>
+        <v>0.11999999999999744</v>
       </c>
       <c r="L7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!L$17</f>
+        <v>0.13999999999999346</v>
       </c>
       <c r="M7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!M$17</f>
+        <v>0.15999999999999659</v>
       </c>
       <c r="N7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!N$17</f>
+        <v>0.17999999999999261</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <f>'Max Biofuel Blends'!O$17</f>
+        <v>0.19999999999999574</v>
       </c>
       <c r="P7">
-        <f t="shared" ref="P7:AH7" si="0">Q7-0.02</f>
-        <v>1.9999999999999938E-2</v>
+        <f>'Max Biofuel Blends'!P$17</f>
+        <v>0.21999999999999176</v>
       </c>
       <c r="Q7">
-        <f t="shared" si="0"/>
-        <v>3.9999999999999938E-2</v>
+        <f>'Max Biofuel Blends'!Q$17</f>
+        <v>0.23999999999999488</v>
       </c>
       <c r="R7">
-        <f t="shared" si="0"/>
-        <v>5.9999999999999942E-2</v>
+        <f>'Max Biofuel Blends'!R$17</f>
+        <v>0.25999999999999801</v>
       </c>
       <c r="S7">
-        <f t="shared" si="0"/>
-        <v>7.9999999999999946E-2</v>
+        <f>'Max Biofuel Blends'!S$17</f>
+        <v>0.27999999999999403</v>
       </c>
       <c r="T7">
-        <f t="shared" si="0"/>
-        <v>9.999999999999995E-2</v>
+        <f>'Max Biofuel Blends'!T$17</f>
+        <v>0.29999999999999716</v>
       </c>
       <c r="U7">
-        <f t="shared" si="0"/>
-        <v>0.11999999999999995</v>
+        <f>'Max Biofuel Blends'!U$17</f>
+        <v>0.31999999999999318</v>
       </c>
       <c r="V7">
-        <f t="shared" si="0"/>
-        <v>0.13999999999999996</v>
+        <f>'Max Biofuel Blends'!V$17</f>
+        <v>0.33999999999999631</v>
       </c>
       <c r="W7">
-        <f t="shared" si="0"/>
-        <v>0.15999999999999995</v>
+        <f>'Max Biofuel Blends'!W$17</f>
+        <v>0.35999999999999233</v>
       </c>
       <c r="X7">
-        <f t="shared" si="0"/>
-        <v>0.17999999999999994</v>
+        <f>'Max Biofuel Blends'!X$17</f>
+        <v>0.37999999999999545</v>
       </c>
       <c r="Y7">
-        <f t="shared" si="0"/>
-        <v>0.19999999999999993</v>
+        <f>'Max Biofuel Blends'!Y$17</f>
+        <v>0.39999999999999858</v>
       </c>
       <c r="Z7">
-        <f t="shared" si="0"/>
-        <v>0.21999999999999992</v>
+        <f>'Max Biofuel Blends'!Z$17</f>
+        <v>0.4199999999999946</v>
       </c>
       <c r="AA7">
-        <f t="shared" si="0"/>
-        <v>0.23999999999999991</v>
+        <f>'Max Biofuel Blends'!AA$17</f>
+        <v>0.43999999999999773</v>
       </c>
       <c r="AB7">
-        <f t="shared" si="0"/>
-        <v>0.2599999999999999</v>
+        <f>'Max Biofuel Blends'!AB$17</f>
+        <v>0.45999999999999375</v>
       </c>
       <c r="AC7">
-        <f t="shared" si="0"/>
-        <v>0.27999999999999992</v>
+        <f>'Max Biofuel Blends'!AC$17</f>
+        <v>0.47999999999999687</v>
       </c>
       <c r="AD7">
-        <f t="shared" si="0"/>
-        <v>0.29999999999999993</v>
+        <f>'Max Biofuel Blends'!AD$17</f>
+        <v>0.49999999999999289</v>
       </c>
       <c r="AE7">
-        <f t="shared" si="0"/>
-        <v>0.31999999999999995</v>
+        <f>'Max Biofuel Blends'!AE$17</f>
+        <v>0.51999999999999602</v>
       </c>
       <c r="AF7">
-        <f t="shared" si="0"/>
-        <v>0.33999999999999997</v>
+        <f>'Max Biofuel Blends'!AF$17</f>
+        <v>0.53999999999999204</v>
       </c>
       <c r="AG7">
-        <f t="shared" si="0"/>
-        <v>0.36</v>
+        <f>'Max Biofuel Blends'!AG$17</f>
+        <v>0.55999999999999517</v>
       </c>
       <c r="AH7">
-        <f>AI7-0.02</f>
-        <v>0.38</v>
+        <f>'Max Biofuel Blends'!AH$17</f>
+        <v>0.57999999999999829</v>
       </c>
       <c r="AI7">
-        <v>0.4</v>
+        <f>'Max Biofuel Blends'!AI$17</f>
+        <v>0.59999999999999432</v>
       </c>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.25">

</xml_diff>